<commit_message>
test cases added for statndard user inventory, cart,checkout
</commit_message>
<xml_diff>
--- a/test-cases/Test cases.xlsx
+++ b/test-cases/Test cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA project\QA_Automation\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AAA0C693-BD62-428B-86BC-30B82D8E7B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2E1B4C-954A-4334-819B-9472D7DFAFB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6C2D49F0-C577-4C83-8AEE-64E5DB6874FD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C2D49F0-C577-4C83-8AEE-64E5DB6874FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="111">
   <si>
     <t>Test Identifier</t>
   </si>
@@ -263,12 +263,201 @@
 4. The password input box displayed masked characters for ""secret_sauce"". (Pass)
 5. No visual distortions were observed during login or page transition.</t>
   </si>
+  <si>
+    <t>Verify Inventory page loads</t>
+  </si>
+  <si>
+    <t>Ensure inventory page loads successfully and products are visible.</t>
+  </si>
+  <si>
+    <t>User is logged in as standard_user and navigated to Inventory page (/inventory.html).</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>1. Login as standard_user with valid password.
+2. Confirm the page title/header shows Products.
+3. Verify product list is displayed on the page.</t>
+  </si>
+  <si>
+    <t>1. User is redirected to https://www.saucedemo.com/inventory.html.
+2. Header Products is visible.
+3. Product items/cards are visible (list is not empty).</t>
+  </si>
+  <si>
+    <t>Add one item to cart</t>
+  </si>
+  <si>
+    <t>Verify adding one product updates button state and cart badge count.</t>
+  </si>
+  <si>
+    <t>User is logged in and on Inventory page.</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>1. Locate product Sauce Labs Backpack.
+2. Click Add to cart for that product.
+3. Observe the cart icon badge (top right).
+4. Observe the button text for the same product.</t>
+  </si>
+  <si>
+    <t>1. Button changes from Add to cart to Remove for Sauce Labs Backpack.
+2. Cart badge appears and shows1.</t>
+  </si>
+  <si>
+    <t>Remove item from cart (Inventory)</t>
+  </si>
+  <si>
+    <t>Verify removing an added product updates button state and cart badge count.</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>Add multiple items to cart</t>
+  </si>
+  <si>
+    <t>Verify cart badge reflects total items added.</t>
+  </si>
+  <si>
+    <t>User is logged in and on Inventory page; cart is empty (no badge).</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>Verify cart contains added items</t>
+  </si>
+  <si>
+    <t>Ensure items added from Inventory are displayed correctly in Cart page.</t>
+  </si>
+  <si>
+    <t>User is logged in; at least 1 item is added to cart (badge &gt; 0).</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Remove item from Cart page</t>
+  </si>
+  <si>
+    <t>Verify removing an item from cart updates cart contents and badge count.</t>
+  </si>
+  <si>
+    <t>User is on Cart page with at least 1 item added.</t>
+  </si>
+  <si>
+    <t>1. Removed item no longer appears in cart list.2. Cart badge decreases by 1 (or disappears if cart becomes empty).</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>Continue Shopping navigation</t>
+  </si>
+  <si>
+    <t>Verify Continue Shopping button navigates back to Inventory page.</t>
+  </si>
+  <si>
+    <t>User is on Cart page.</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>Complete checkout for one item</t>
+  </si>
+  <si>
+    <t>Verify a user can successfully place an order using checkout flow.</t>
+  </si>
+  <si>
+    <t>User is logged in; at least 1 item is added to cart; user is on Cart page.</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>Checkout form validation</t>
+  </si>
+  <si>
+    <t>Verify appropriate error message is shown when required checkout fields are missing.</t>
+  </si>
+  <si>
+    <t>User is logged in; at least 1 item added; user is on Cart page.</t>
+  </si>
+  <si>
+    <t>1. User remains on Checkout Information page.2. Error message is displayed indicating missing First Name (or required field).3. User should not proceed to Overview page.</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>Sort products by price low to high</t>
+  </si>
+  <si>
+    <t>Verify the sort dropdown sorts items by price in ascending order.</t>
+  </si>
+  <si>
+    <t>1. Products reorder based on increasing price.2. The first displayed item should have the lowest price and the last item the highest price.</t>
+  </si>
+  <si>
+    <t>1. User navigates to https://www.saucedemo.com/cart.html.2. Added item(s) appear in the cart list.3. Item name(s) and price(s) match the Inventory page.4. Remove button is visible for each item.</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>User is logged in and on Inventory page with Sauce Labs Backpack already added to cart (badge = 1).</t>
+  </si>
+  <si>
+    <t>1. Click Add to cart for Sauce Labs Backpack.2. Click Add to cart for Sauce Labs Bike Light.3. Click Add to cart for Sauce Labs Bolt T-Shirt.4. Observe cart badge count.</t>
+  </si>
+  <si>
+    <t>1. Each selected product button changes to Remove.2. Cart badge updates to 3.</t>
+  </si>
+  <si>
+    <t>1. Click the cart icon (top right).2. Verify Cart page loads.3. Verify added item(s) are listed with correct name and price.4. Verify Remove button is available for each item.</t>
+  </si>
+  <si>
+    <t>1. On Cart page, click Remove for one item.2. Observe cart list after removal.3. Observe cart badge count (top right).</t>
+  </si>
+  <si>
+    <t>1. Click Continue Shopping.2. Observe navigation URL and page header.</t>
+  </si>
+  <si>
+    <t>1. User is redirected to https://www.saucedemo.com/inventory.html.2. Header Products is visible again.</t>
+  </si>
+  <si>
+    <t>1. Click Checkout.2. Enter First Name: Test.3. Enter Last Name: User.4. Enter Zip/Postal Code: 12345.5. Click Continue.6. Verify Overview page loads.7. Click Finish.</t>
+  </si>
+  <si>
+    <t>1. User navigates to Checkout Information page.2. After Continue, user navigates to Checkout Overview page.3. Order summary is displayed (items, totals).4. After Finish, confirmation page is displayed with success message (e.g., Thank you for your order!).</t>
+  </si>
+  <si>
+    <t>1. Click Checkout.2. Leave First Name empty.3. Enter Last Name: User.4. Enter Zip/Postal Code: 12345.5. Click Continue.</t>
+  </si>
+  <si>
+    <t>1. On Inventory page, open Sort dropdown (top right).2. Select Price (low to high).3. Observe product prices shown in list order.</t>
+  </si>
+  <si>
+    <t>1. On Inventory page, locate Sauce Labs Backpack.
+2. Click Remove.
+3. Observe cart badge.
+4. Observe button text again.</t>
+  </si>
+  <si>
+    <t>1. Button changes from Remove back to Add to cart.
+2. Cart badge decreases accordingly (badge disappears if cart is empty).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -277,21 +466,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -314,7 +511,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -386,31 +583,118 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -418,6 +702,25 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="14">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -432,6 +735,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -466,28 +770,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -496,8 +783,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -514,10 +799,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -528,8 +814,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -546,6 +830,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -555,7 +840,7 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -566,8 +851,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -584,10 +867,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -598,8 +882,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -616,10 +898,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -630,8 +913,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -648,10 +929,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -662,8 +944,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -680,10 +960,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -694,8 +975,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -712,10 +991,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -726,8 +1006,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -744,10 +1022,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -758,8 +1037,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -776,10 +1053,11 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
@@ -790,8 +1068,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -808,6 +1084,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -817,7 +1094,7 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right style="thin">
           <color rgb="FF000000"/>
@@ -826,8 +1103,6 @@
           <color rgb="FF000000"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -860,7 +1135,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8796CFEC-F437-4BF2-A6E7-9F7370BD9B4D}" name="Table2" displayName="Table2" ref="A1:K5" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" tableBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8796CFEC-F437-4BF2-A6E7-9F7370BD9B4D}" name="Table2" displayName="Table2" ref="A1:K5" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" tableBorderDxfId="13">
   <autoFilter ref="A1:K5" xr:uid="{8796CFEC-F437-4BF2-A6E7-9F7370BD9B4D}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{5633DDAE-E13E-41BC-9926-ABE907AA412A}" name="Test Identifier" dataDxfId="12"/>
@@ -1196,272 +1471,606 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4B7A3A-D8ED-482A-B3B0-9C9C7FD43AA9}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K55"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="32.88671875" customWidth="1"/>
-    <col min="4" max="4" width="27.44140625" customWidth="1"/>
-    <col min="5" max="5" width="38.21875" customWidth="1"/>
-    <col min="6" max="6" width="51.77734375" customWidth="1"/>
-    <col min="7" max="7" width="53" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" customWidth="1"/>
-    <col min="9" max="9" width="9.21875" customWidth="1"/>
-    <col min="10" max="10" width="15.88671875" customWidth="1"/>
-    <col min="11" max="11" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="16" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="27.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="38.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="53" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.77734375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="11" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="218.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="218.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="202.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="234" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="13" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="8" spans="1:11" s="6" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="8" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" s="8" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="7"/>
+    </row>
+    <row r="14" spans="1:11" s="8" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" s="8" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="7"/>
+    </row>
+    <row r="16" spans="1:11" s="8" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="7"/>
+    </row>
+    <row r="17" spans="1:11" s="8" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K17" s="7"/>
+    </row>
+    <row r="18" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="33" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="34" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="35" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="36" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="37" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="38" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="40" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="41" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="42" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="43" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="44" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="45" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="46" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="47" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="48" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="49" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="50" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="51" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="52" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="53" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="54" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="55" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>